<commit_message>
AMBUb.CO STD + Excel
</commit_message>
<xml_diff>
--- a/data/cox_xlsx/AMBUb.CO.xlsx
+++ b/data/cox_xlsx/AMBUb.CO.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="459">
   <si>
     <t>Company Fundamentals - Income Statement</t>
   </si>
@@ -825,7 +825,13 @@
     <t>Current liabilities</t>
   </si>
   <si>
+    <t>Interest-bearing debt (do not use)</t>
+  </si>
+  <si>
     <t>Other interest-bearing debt</t>
+  </si>
+  <si>
+    <t>Corporate bonds (do not use)</t>
   </si>
   <si>
     <t>Borrowings</t>
@@ -13549,9 +13555,7 @@
       <c r="I85" s="19">
         <v>0.0</v>
       </c>
-      <c r="J85" s="15">
-        <v>884.63</v>
-      </c>
+      <c r="J85" s="15"/>
       <c r="K85" s="19"/>
       <c r="L85" s="19"/>
       <c r="M85" s="19"/>
@@ -13972,8 +13976,8 @@
       </c>
     </row>
     <row r="93" ht="15.0" customHeight="1">
-      <c r="A93" s="14" t="s">
-        <v>259</v>
+      <c r="A93" s="27" t="s">
+        <v>268</v>
       </c>
       <c r="B93" s="19"/>
       <c r="C93" s="19"/>
@@ -14029,7 +14033,7 @@
     </row>
     <row r="94" ht="15.0" customHeight="1">
       <c r="A94" s="14" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B94" s="19"/>
       <c r="C94" s="19"/>
@@ -14058,8 +14062,8 @@
       <c r="V94" s="19"/>
     </row>
     <row r="95" ht="15.0" customHeight="1">
-      <c r="A95" s="14" t="s">
-        <v>261</v>
+      <c r="A95" s="27" t="s">
+        <v>270</v>
       </c>
       <c r="B95" s="19"/>
       <c r="C95" s="19"/>
@@ -14143,7 +14147,7 @@
     </row>
     <row r="97" ht="15.0" customHeight="1">
       <c r="A97" s="14" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B97" s="18">
         <v>7.85</v>
@@ -14195,7 +14199,7 @@
     </row>
     <row r="98" ht="15.0" customHeight="1">
       <c r="A98" s="14" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B98" s="18">
         <v>17.26</v>
@@ -14349,7 +14353,7 @@
     </row>
     <row r="101" ht="15.0" customHeight="1">
       <c r="A101" s="14" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B101" s="19"/>
       <c r="C101" s="19"/>
@@ -14377,7 +14381,7 @@
     </row>
     <row r="102" ht="15.0" customHeight="1">
       <c r="A102" s="16" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B102" s="17">
         <v>754.9</v>
@@ -14445,7 +14449,7 @@
     </row>
     <row r="103" ht="15.0" customHeight="1">
       <c r="A103" s="16" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B103" s="17">
         <v>2573.89</v>
@@ -14513,7 +14517,7 @@
     </row>
     <row r="104" ht="15.0" customHeight="1">
       <c r="A104" s="14" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B104" s="15">
         <v>211.87</v>
@@ -14581,7 +14585,7 @@
     </row>
     <row r="105" ht="15.0" customHeight="1">
       <c r="A105" s="14" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B105" s="15">
         <v>9259.72</v>
@@ -14649,7 +14653,7 @@
     </row>
     <row r="106" ht="15.0" customHeight="1">
       <c r="A106" s="14" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B106" s="19"/>
       <c r="C106" s="19"/>
@@ -14701,7 +14705,7 @@
     </row>
     <row r="107" ht="15.0" customHeight="1">
       <c r="A107" s="14" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B107" s="19"/>
       <c r="C107" s="19"/>
@@ -14761,7 +14765,7 @@
     </row>
     <row r="108" ht="15.0" customHeight="1">
       <c r="A108" s="14" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B108" s="18">
         <v>56.5</v>
@@ -14829,7 +14833,7 @@
     </row>
     <row r="109" ht="15.0" customHeight="1">
       <c r="A109" s="14" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B109" s="19"/>
       <c r="C109" s="15">
@@ -14895,7 +14899,7 @@
     </row>
     <row r="110" ht="15.0" customHeight="1">
       <c r="A110" s="14" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B110" s="15">
         <v>9203.22</v>
@@ -14943,7 +14947,7 @@
     </row>
     <row r="111" ht="15.0" customHeight="1">
       <c r="A111" s="14" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B111" s="19"/>
       <c r="C111" s="19"/>
@@ -14975,7 +14979,7 @@
     </row>
     <row r="112" ht="15.0" customHeight="1">
       <c r="A112" s="16" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B112" s="17">
         <v>9471.59</v>
@@ -15043,7 +15047,7 @@
     </row>
     <row r="113" ht="15.0" customHeight="1">
       <c r="A113" s="14" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B113" s="19"/>
       <c r="C113" s="19"/>
@@ -15075,7 +15079,7 @@
     </row>
     <row r="114" ht="15.0" customHeight="1">
       <c r="A114" s="16" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B114" s="17">
         <v>9471.59</v>
@@ -15143,7 +15147,7 @@
     </row>
     <row r="115" ht="15.0" customHeight="1">
       <c r="A115" s="14" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B115" s="19"/>
       <c r="C115" s="19"/>
@@ -15173,7 +15177,7 @@
     </row>
     <row r="116" ht="15.0" customHeight="1">
       <c r="A116" s="16" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B116" s="26">
         <v>12045.48</v>
@@ -15241,7 +15245,7 @@
     </row>
     <row r="117" ht="15.0" customHeight="1">
       <c r="A117" s="14" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B117" s="18">
         <v>2.74</v>
@@ -15309,7 +15313,7 @@
     </row>
     <row r="118" ht="15.0" customHeight="1">
       <c r="A118" s="14" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B118" s="15">
         <v>269.29</v>
@@ -15377,7 +15381,7 @@
     </row>
     <row r="119" ht="15.0" customHeight="1">
       <c r="A119" s="14" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B119" s="15">
         <v>266.56</v>
@@ -15445,7 +15449,7 @@
     </row>
     <row r="120" ht="15.0" customHeight="1">
       <c r="A120" s="14" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B120" s="19"/>
       <c r="C120" s="19"/>
@@ -15497,7 +15501,7 @@
     </row>
     <row r="121" ht="15.0" customHeight="1">
       <c r="A121" s="14" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B121" s="19"/>
       <c r="C121" s="19"/>
@@ -15545,7 +15549,7 @@
     </row>
     <row r="122" ht="15.0" customHeight="1">
       <c r="A122" s="14" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B122" s="19"/>
       <c r="C122" s="19"/>
@@ -15595,7 +15599,7 @@
     </row>
     <row r="123" ht="15.0" customHeight="1">
       <c r="A123" s="14" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B123" s="19"/>
       <c r="C123" s="19"/>
@@ -15639,7 +15643,7 @@
     </row>
     <row r="124" ht="15.0" customHeight="1">
       <c r="A124" s="14" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B124" s="19"/>
       <c r="C124" s="19"/>
@@ -15667,7 +15671,7 @@
     </row>
     <row r="125" ht="15.0" customHeight="1">
       <c r="A125" s="14" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B125" s="19"/>
       <c r="C125" s="19"/>
@@ -15699,7 +15703,7 @@
     </row>
     <row r="126" ht="15.0" customHeight="1">
       <c r="A126" s="14" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B126" s="19"/>
       <c r="C126" s="19"/>
@@ -15747,7 +15751,7 @@
     </row>
     <row r="127" ht="15.0" customHeight="1">
       <c r="A127" s="14" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B127" s="19"/>
       <c r="C127" s="19"/>
@@ -15779,7 +15783,7 @@
     </row>
     <row r="128" ht="15.0" customHeight="1">
       <c r="A128" s="14" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B128" s="15">
         <v>128.69</v>
@@ -15831,7 +15835,7 @@
     </row>
     <row r="129" ht="15.0" customHeight="1">
       <c r="A129" s="14" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B129" s="15">
         <v>384.51</v>
@@ -15883,7 +15887,7 @@
     </row>
     <row r="130" ht="15.0" customHeight="1">
       <c r="A130" s="14" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B130" s="15">
         <v>654.46</v>
@@ -15935,7 +15939,7 @@
     </row>
     <row r="131" ht="15.0" customHeight="1">
       <c r="A131" s="14" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B131" s="19"/>
       <c r="C131" s="19"/>
@@ -15965,7 +15969,7 @@
     </row>
     <row r="132" ht="15.0" customHeight="1">
       <c r="A132" s="14" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B132" s="19"/>
       <c r="C132" s="19"/>
@@ -15997,7 +16001,7 @@
     </row>
     <row r="133" ht="15.0" customHeight="1">
       <c r="A133" s="14" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B133" s="15">
         <v>1569.44</v>
@@ -16033,7 +16037,7 @@
     </row>
     <row r="134" ht="15.0" customHeight="1">
       <c r="A134" s="14" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B134" s="19"/>
       <c r="C134" s="19"/>
@@ -16103,7 +16107,7 @@
     </row>
     <row r="136" ht="15.0" customHeight="1">
       <c r="A136" s="14" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B136" s="28"/>
       <c r="C136" s="28"/>
@@ -16143,7 +16147,7 @@
     </row>
     <row r="137" ht="15.0" customHeight="1">
       <c r="A137" s="14" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B137" s="15">
         <v>232.24</v>
@@ -16211,7 +16215,7 @@
     </row>
     <row r="138" ht="15.0" customHeight="1">
       <c r="A138" s="14" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B138" s="15">
         <v>234.97</v>
@@ -16279,7 +16283,7 @@
     </row>
     <row r="139" ht="15.0" customHeight="1">
       <c r="A139" s="14" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B139" s="18">
         <v>0.87</v>
@@ -16347,7 +16351,7 @@
     </row>
     <row r="140" ht="15.0" customHeight="1">
       <c r="A140" s="14" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B140" s="18">
         <v>2.74</v>
@@ -16415,7 +16419,7 @@
     </row>
     <row r="141" ht="15.0" customHeight="1">
       <c r="A141" s="14" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B141" s="18">
         <v>34.32</v>
@@ -16481,7 +16485,7 @@
     </row>
     <row r="142" ht="15.0" customHeight="1">
       <c r="A142" s="14" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B142" s="18">
         <v>34.32</v>
@@ -16547,7 +16551,7 @@
     </row>
     <row r="143" ht="15.0" customHeight="1">
       <c r="A143" s="14" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B143" s="18">
         <v>0.13</v>
@@ -17489,7 +17493,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -17862,67 +17866,67 @@
         <v>43</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="R15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="T15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="V15" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1" outlineLevel="1">
@@ -17995,7 +17999,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -18089,7 +18093,7 @@
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="14" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B20" s="15">
         <v>955.82</v>
@@ -18157,7 +18161,7 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="14" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B21" s="23">
         <v>-158.52</v>
@@ -18225,7 +18229,7 @@
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="14" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B22" s="19"/>
       <c r="C22" s="19"/>
@@ -18269,7 +18273,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="14" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B23" s="18">
         <v>45.52</v>
@@ -18331,7 +18335,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B24" s="20">
         <v>-43.95</v>
@@ -18363,7 +18367,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="14" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B25" s="20">
         <v>-14.13</v>
@@ -18397,7 +18401,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="14" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B26" s="23">
         <v>-428.47</v>
@@ -18451,7 +18455,7 @@
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="14" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B27" s="23">
         <v>-395.51</v>
@@ -18517,7 +18521,7 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="14" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B28" s="23">
         <v>-167.94</v>
@@ -18583,7 +18587,7 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="14" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B29" s="15">
         <v>134.98</v>
@@ -18631,7 +18635,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="14" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B30" s="19"/>
       <c r="C30" s="19"/>
@@ -18675,7 +18679,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="14" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
@@ -18723,7 +18727,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="14" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B32" s="19"/>
       <c r="C32" s="19"/>
@@ -18763,7 +18767,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="14" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B33" s="18">
         <v>48.65</v>
@@ -18813,7 +18817,7 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="14" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B34" s="15">
         <v>583.85</v>
@@ -18867,7 +18871,7 @@
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="14" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B35" s="15">
         <v>343.72</v>
@@ -18897,7 +18901,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="14" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B36" s="15">
         <v>128.7</v>
@@ -18927,7 +18931,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="14" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B37" s="15">
         <v>108.3</v>
@@ -18957,7 +18961,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="14" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B38" s="18">
         <v>3.14</v>
@@ -18987,7 +18991,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="14" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B39" s="19">
         <v>0.0</v>
@@ -19017,7 +19021,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="14" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B40" s="19"/>
       <c r="C40" s="19"/>
@@ -19049,7 +19053,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="14" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B41" s="19"/>
       <c r="C41" s="19"/>
@@ -19149,7 +19153,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="14" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B44" s="19"/>
       <c r="C44" s="19"/>
@@ -19189,7 +19193,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="14" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B45" s="19"/>
       <c r="C45" s="19"/>
@@ -19237,7 +19241,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="14" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B46" s="19"/>
       <c r="C46" s="19"/>
@@ -19281,7 +19285,7 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="14" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B47" s="18">
         <v>23.54</v>
@@ -19311,7 +19315,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="14" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B48" s="19"/>
       <c r="C48" s="19"/>
@@ -19339,7 +19343,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="14" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B49" s="15">
         <v>229.15</v>
@@ -19371,7 +19375,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="14" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B50" s="19"/>
       <c r="C50" s="19"/>
@@ -19403,7 +19407,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="14" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B51" s="19"/>
       <c r="C51" s="19"/>
@@ -19433,7 +19437,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B52" s="19"/>
       <c r="C52" s="19"/>
@@ -19463,7 +19467,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="14" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B53" s="19"/>
       <c r="C53" s="19"/>
@@ -19493,7 +19497,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="16" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B54" s="17">
         <v>1241.47</v>
@@ -19561,7 +19565,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="14" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B55" s="23">
         <v>-419.06</v>
@@ -19609,7 +19613,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="14" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B56" s="23">
         <v>-183.63</v>
@@ -19649,7 +19653,7 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="14" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B57" s="19"/>
       <c r="C57" s="19"/>
@@ -19689,7 +19693,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="14" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B58" s="19"/>
       <c r="C58" s="19"/>
@@ -19729,7 +19733,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="14" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B59" s="19"/>
       <c r="C59" s="19"/>
@@ -19771,7 +19775,7 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="14" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B60" s="19"/>
       <c r="C60" s="19"/>
@@ -19807,7 +19811,7 @@
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="14" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B61" s="19"/>
       <c r="C61" s="19"/>
@@ -19853,7 +19857,7 @@
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="14" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B62" s="19"/>
       <c r="C62" s="19"/>
@@ -19911,7 +19915,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="14" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B63" s="19"/>
       <c r="C63" s="19"/>
@@ -19951,7 +19955,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="16" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B64" s="24">
         <v>-602.69</v>
@@ -20019,7 +20023,7 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="14" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B65" s="19"/>
       <c r="C65" s="19"/>
@@ -20059,7 +20063,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="14" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B66" s="19"/>
       <c r="C66" s="19"/>
@@ -20091,7 +20095,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="14" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B67" s="19"/>
       <c r="C67" s="19"/>
@@ -20123,7 +20127,7 @@
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="14" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B68" s="19"/>
       <c r="C68" s="19">
@@ -20167,7 +20171,7 @@
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="14" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B69" s="19"/>
       <c r="C69" s="19">
@@ -20209,7 +20213,7 @@
     </row>
     <row r="70" ht="15.0" customHeight="1">
       <c r="A70" s="14" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B70" s="19"/>
       <c r="C70" s="19"/>
@@ -20241,7 +20245,7 @@
     </row>
     <row r="71" ht="15.0" customHeight="1">
       <c r="A71" s="14" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B71" s="20">
         <v>-98.88</v>
@@ -20279,7 +20283,7 @@
     </row>
     <row r="72" ht="15.0" customHeight="1">
       <c r="A72" s="14" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B72" s="19"/>
       <c r="C72" s="19"/>
@@ -20309,7 +20313,7 @@
     </row>
     <row r="73" ht="15.0" customHeight="1">
       <c r="A73" s="14" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B73" s="19"/>
       <c r="C73" s="19"/>
@@ -20341,7 +20345,7 @@
     </row>
     <row r="74" ht="15.0" customHeight="1">
       <c r="A74" s="14" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B74" s="19"/>
       <c r="C74" s="19"/>
@@ -20373,7 +20377,7 @@
     </row>
     <row r="75" ht="15.0" customHeight="1">
       <c r="A75" s="14" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B75" s="18">
         <v>17.26</v>
@@ -20429,7 +20433,7 @@
     </row>
     <row r="76" ht="15.0" customHeight="1">
       <c r="A76" s="14" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B76" s="19"/>
       <c r="C76" s="19"/>
@@ -20481,7 +20485,7 @@
     </row>
     <row r="77" ht="15.0" customHeight="1">
       <c r="A77" s="14" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B77" s="19"/>
       <c r="C77" s="19">
@@ -20523,7 +20527,7 @@
     </row>
     <row r="78" ht="15.0" customHeight="1">
       <c r="A78" s="14" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B78" s="23">
         <v>-160.09</v>
@@ -20589,7 +20593,7 @@
     </row>
     <row r="79" ht="15.0" customHeight="1">
       <c r="A79" s="14" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B79" s="18">
         <v>1.57</v>
@@ -20617,7 +20621,7 @@
     </row>
     <row r="80" ht="15.0" customHeight="1">
       <c r="A80" s="14" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B80" s="19"/>
       <c r="C80" s="19"/>
@@ -20659,7 +20663,7 @@
     </row>
     <row r="81" ht="15.0" customHeight="1">
       <c r="A81" s="14" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B81" s="19"/>
       <c r="C81" s="19">
@@ -20717,7 +20721,7 @@
     </row>
     <row r="82" ht="15.0" customHeight="1">
       <c r="A82" s="14" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B82" s="19"/>
       <c r="C82" s="19"/>
@@ -20751,7 +20755,7 @@
     </row>
     <row r="83" ht="15.0" customHeight="1">
       <c r="A83" s="14" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B83" s="19"/>
       <c r="C83" s="19"/>
@@ -20791,7 +20795,7 @@
     </row>
     <row r="84" ht="15.0" customHeight="1">
       <c r="A84" s="14" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B84" s="19"/>
       <c r="C84" s="19"/>
@@ -20823,7 +20827,7 @@
     </row>
     <row r="85" ht="15.0" customHeight="1">
       <c r="A85" s="14" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B85" s="19"/>
       <c r="C85" s="19"/>
@@ -20851,7 +20855,7 @@
     </row>
     <row r="86" ht="15.0" customHeight="1">
       <c r="A86" s="14" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B86" s="19"/>
       <c r="C86" s="19"/>
@@ -20879,7 +20883,7 @@
     </row>
     <row r="87" ht="15.0" customHeight="1">
       <c r="A87" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B87" s="24">
         <v>-240.13</v>
@@ -20947,7 +20951,7 @@
     </row>
     <row r="88" ht="15.0" customHeight="1">
       <c r="A88" s="14" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B88" s="20">
         <v>-4.71</v>
@@ -21013,7 +21017,7 @@
     </row>
     <row r="89" ht="15.0" customHeight="1">
       <c r="A89" s="14" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B89" s="15">
         <v>965.21</v>
@@ -21149,7 +21153,7 @@
     </row>
     <row r="91" ht="15.0" customHeight="1">
       <c r="A91" s="14" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B91" s="15">
         <v>398.65</v>
@@ -21205,7 +21209,7 @@
     </row>
     <row r="92" ht="15.0" customHeight="1">
       <c r="A92" s="14" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B92" s="19"/>
       <c r="C92" s="19"/>
@@ -21233,7 +21237,7 @@
     </row>
     <row r="93" ht="15.0" customHeight="1">
       <c r="A93" s="16" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B93" s="17">
         <v>393.94</v>
@@ -21301,7 +21305,7 @@
     </row>
     <row r="94" ht="15.0" customHeight="1">
       <c r="A94" s="14" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B94" s="19"/>
       <c r="C94" s="19"/>
@@ -21333,7 +21337,7 @@
     </row>
     <row r="95" ht="15.0" customHeight="1">
       <c r="A95" s="14" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B95" s="15">
         <v>638.79</v>
@@ -22293,7 +22297,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -22466,31 +22470,31 @@
         <v>38</v>
       </c>
       <c r="W11" s="7" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="X11" s="7" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="Y11" s="7" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="Z11" s="7" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="AA11" s="7" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="AB11" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="AC11" s="7" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="AD11" s="7" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="AE11" s="7" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="1" outlineLevel="1">
@@ -22861,16 +22865,16 @@
         <v>44</v>
       </c>
       <c r="AB15" s="10" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="AD15" s="10" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="AE15" s="10" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1" outlineLevel="1">
@@ -22970,7 +22974,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -23071,36 +23075,36 @@
         <v>68</v>
       </c>
       <c r="W19" s="13" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="X19" s="13" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="Y19" s="13" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="Z19" s="13" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="AA19" s="13" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="AB19" s="13" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="AC19" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="AD19" s="13" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="AE19" s="13" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="29" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B20" s="30"/>
       <c r="C20" s="30"/>
@@ -23135,7 +23139,7 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="31" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B21" s="32">
         <v>38636.02</v>
@@ -23230,7 +23234,7 @@
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="31" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B22" s="32">
         <v>46661.22</v>
@@ -23317,7 +23321,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="29" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B23" s="30"/>
       <c r="C23" s="30"/>
@@ -23352,7 +23356,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="31" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B24" s="32">
         <v>39136.68</v>
@@ -23447,7 +23451,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="31" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B25" s="32">
         <v>45886.54</v>
@@ -23534,7 +23538,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="29" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B26" s="30"/>
       <c r="C26" s="30"/>
@@ -23569,7 +23573,7 @@
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="31" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B27" s="33">
         <v>145.33</v>
@@ -23664,7 +23668,7 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="31" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B28" s="33">
         <v>173.86</v>
@@ -23751,7 +23755,7 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="29" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B29" s="30"/>
       <c r="C29" s="30"/>
@@ -23786,7 +23790,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="31" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B30" s="35">
         <v>1.65</v>
@@ -23879,7 +23883,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="31" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B31" s="35">
         <v>0.25</v>
@@ -23956,7 +23960,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="29" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B32" s="30"/>
       <c r="C32" s="30"/>
@@ -23991,7 +23995,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="31" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B33" s="35">
         <v>0.41</v>
@@ -24086,7 +24090,7 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="31" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B34" s="35">
         <v>0.17</v>
@@ -24173,7 +24177,7 @@
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="31" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B35" s="35">
         <v>0.41</v>
@@ -24268,7 +24272,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="31" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B36" s="35">
         <v>0.17</v>
@@ -24355,7 +24359,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="29" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B37" s="30"/>
       <c r="C37" s="30"/>
@@ -24390,7 +24394,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="31" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B38" s="34">
         <v>4.09</v>
@@ -24485,7 +24489,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="31" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B39" s="34">
         <v>5.76</v>
@@ -24572,7 +24576,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="29" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B40" s="30"/>
       <c r="C40" s="30"/>
@@ -24607,7 +24611,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="31" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B41" s="34">
         <v>8.86</v>
@@ -24688,7 +24692,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="31" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B42" s="34">
         <v>17.56</v>
@@ -24761,7 +24765,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="29" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B43" s="30"/>
       <c r="C43" s="30"/>
@@ -24796,7 +24800,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="31" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B44" s="34">
         <v>4.09</v>
@@ -24891,7 +24895,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="31" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B45" s="34">
         <v>5.85</v>
@@ -24978,7 +24982,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="29" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B46" s="30"/>
       <c r="C46" s="30"/>
@@ -25013,7 +25017,7 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="31" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B47" s="34">
         <v>60.63</v>
@@ -25100,7 +25104,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="31" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B48" s="33">
         <v>397.85</v>
@@ -25171,7 +25175,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="29" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B49" s="30"/>
       <c r="C49" s="30"/>
@@ -25206,7 +25210,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="31" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B50" s="34">
         <v>25.2</v>
@@ -25301,7 +25305,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="31" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B51" s="34">
         <v>51.5</v>
@@ -25388,7 +25392,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="29" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B52" s="30"/>
       <c r="C52" s="30"/>
@@ -25423,7 +25427,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="31" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B53" s="34">
         <v>40.52</v>
@@ -25518,7 +25522,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="31" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B54" s="33">
         <v>107.34</v>
@@ -25605,7 +25609,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="29" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B55" s="30"/>
       <c r="C55" s="30"/>
@@ -25640,7 +25644,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="31" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B56" s="34">
         <v>40.52</v>
@@ -25735,7 +25739,7 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="31" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B57" s="34">
         <v>5.76</v>
@@ -25822,7 +25826,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="29" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B58" s="30"/>
       <c r="C58" s="30"/>
@@ -25857,7 +25861,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="31" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B59" s="34">
         <v>0.25</v>
@@ -25950,7 +25954,7 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="31" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B60" s="34">
         <v>5.8</v>
@@ -26035,7 +26039,7 @@
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="29" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B61" s="30"/>
       <c r="C61" s="30"/>
@@ -26070,7 +26074,7 @@
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="31" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B62" s="34">
         <v>4.08</v>
@@ -26165,7 +26169,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="31" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B63" s="34">
         <v>6.03</v>
@@ -26252,7 +26256,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="29" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B64" s="30"/>
       <c r="C64" s="30"/>
@@ -26287,7 +26291,7 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="31" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B65" s="34">
         <v>21.33</v>
@@ -26382,7 +26386,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="31" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B66" s="34">
         <v>39.49</v>
@@ -26469,7 +26473,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="29" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B67" s="30"/>
       <c r="C67" s="30"/>
@@ -26504,7 +26508,7 @@
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="31" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B68" s="34">
         <v>31.12</v>
@@ -26599,7 +26603,7 @@
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="31" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B69" s="34">
         <v>58.41</v>
@@ -26686,7 +26690,7 @@
     </row>
     <row r="70" ht="15.0" customHeight="1">
       <c r="A70" s="29" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B70" s="30"/>
       <c r="C70" s="30"/>
@@ -26721,7 +26725,7 @@
     </row>
     <row r="71" ht="15.0" customHeight="1">
       <c r="A71" s="31" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B71" s="34">
         <v>60.49</v>
@@ -26808,7 +26812,7 @@
     </row>
     <row r="72" ht="15.0" customHeight="1">
       <c r="A72" s="31" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B72" s="33">
         <v>367.96</v>

</xml_diff>